<commit_message>
Make IEEE 118 dynamically realistic (low-inertia + bigger disturbances)
The default round-rotor H=4 made the 118 grid too stiff to be interesting
(RoCoF ~0.004 Hz/s). Rebuild at H=2.5 -- modelling the low-inertia condition the
thesis targets -- and widen the load-step disturbance (1.15-1.6x). Result: the
grid now swings meaningfully (mean |RoCoF| 0.0036 -> 0.0102 Hz/s; tail reaches
0.21 Hz/s and Df 0.44 Hz, approaching the 0.8 Hz limit). builder now takes
--target-H / --out. Partial #12: dynamics realistic; PTDF/N-1 network layer for
118 remains.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_generation/andes_cases/ieee118_ibrs.xlsx
+++ b/data_generation/andes_cases/ieee118_ibrs.xlsx
@@ -29195,7 +29195,7 @@
         <v>0</v>
       </c>
       <c r="M2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -29287,7 +29287,7 @@
         <v>0</v>
       </c>
       <c r="M3">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -29379,7 +29379,7 @@
         <v>0</v>
       </c>
       <c r="M4">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -29471,7 +29471,7 @@
         <v>0</v>
       </c>
       <c r="M5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -29563,7 +29563,7 @@
         <v>0</v>
       </c>
       <c r="M6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -29655,7 +29655,7 @@
         <v>0</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -29747,7 +29747,7 @@
         <v>0</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -29839,7 +29839,7 @@
         <v>0</v>
       </c>
       <c r="M9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -29931,7 +29931,7 @@
         <v>0</v>
       </c>
       <c r="M10">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -30023,7 +30023,7 @@
         <v>0</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -30115,7 +30115,7 @@
         <v>0</v>
       </c>
       <c r="M12">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -30207,7 +30207,7 @@
         <v>0</v>
       </c>
       <c r="M13">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -30299,7 +30299,7 @@
         <v>0</v>
       </c>
       <c r="M14">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -30391,7 +30391,7 @@
         <v>0</v>
       </c>
       <c r="M15">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -30483,7 +30483,7 @@
         <v>0</v>
       </c>
       <c r="M16">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N16">
         <v>0</v>
@@ -30575,7 +30575,7 @@
         <v>0</v>
       </c>
       <c r="M17">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -30667,7 +30667,7 @@
         <v>0</v>
       </c>
       <c r="M18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -30759,7 +30759,7 @@
         <v>0</v>
       </c>
       <c r="M19">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -30851,7 +30851,7 @@
         <v>0</v>
       </c>
       <c r="M20">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -30943,7 +30943,7 @@
         <v>0</v>
       </c>
       <c r="M21">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -31035,7 +31035,7 @@
         <v>0</v>
       </c>
       <c r="M22">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -31127,7 +31127,7 @@
         <v>0</v>
       </c>
       <c r="M23">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -31219,7 +31219,7 @@
         <v>0</v>
       </c>
       <c r="M24">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -31311,7 +31311,7 @@
         <v>0</v>
       </c>
       <c r="M25">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N25">
         <v>0</v>
@@ -31403,7 +31403,7 @@
         <v>0</v>
       </c>
       <c r="M26">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N26">
         <v>0</v>
@@ -31495,7 +31495,7 @@
         <v>0</v>
       </c>
       <c r="M27">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -31587,7 +31587,7 @@
         <v>0</v>
       </c>
       <c r="M28">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -31679,7 +31679,7 @@
         <v>0</v>
       </c>
       <c r="M29">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N29">
         <v>0</v>
@@ -31771,7 +31771,7 @@
         <v>0</v>
       </c>
       <c r="M30">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -31863,7 +31863,7 @@
         <v>0</v>
       </c>
       <c r="M31">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -31955,7 +31955,7 @@
         <v>0</v>
       </c>
       <c r="M32">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -32047,7 +32047,7 @@
         <v>0</v>
       </c>
       <c r="M33">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N33">
         <v>0</v>
@@ -32139,7 +32139,7 @@
         <v>0</v>
       </c>
       <c r="M34">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N34">
         <v>0</v>
@@ -32231,7 +32231,7 @@
         <v>0</v>
       </c>
       <c r="M35">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N35">
         <v>0</v>
@@ -32323,7 +32323,7 @@
         <v>0</v>
       </c>
       <c r="M36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N36">
         <v>0</v>
@@ -32415,7 +32415,7 @@
         <v>0</v>
       </c>
       <c r="M37">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N37">
         <v>0</v>
@@ -32507,7 +32507,7 @@
         <v>0</v>
       </c>
       <c r="M38">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N38">
         <v>0</v>
@@ -32599,7 +32599,7 @@
         <v>0</v>
       </c>
       <c r="M39">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N39">
         <v>0</v>
@@ -32691,7 +32691,7 @@
         <v>0</v>
       </c>
       <c r="M40">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N40">
         <v>0</v>
@@ -32783,7 +32783,7 @@
         <v>0</v>
       </c>
       <c r="M41">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N41">
         <v>0</v>
@@ -32875,7 +32875,7 @@
         <v>0</v>
       </c>
       <c r="M42">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N42">
         <v>0</v>
@@ -32967,7 +32967,7 @@
         <v>0</v>
       </c>
       <c r="M43">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N43">
         <v>0</v>
@@ -33059,7 +33059,7 @@
         <v>0</v>
       </c>
       <c r="M44">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N44">
         <v>0</v>
@@ -33151,7 +33151,7 @@
         <v>0</v>
       </c>
       <c r="M45">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N45">
         <v>0</v>
@@ -33243,7 +33243,7 @@
         <v>0</v>
       </c>
       <c r="M46">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N46">
         <v>0</v>
@@ -33335,7 +33335,7 @@
         <v>0</v>
       </c>
       <c r="M47">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N47">
         <v>0</v>
@@ -33427,7 +33427,7 @@
         <v>0</v>
       </c>
       <c r="M48">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N48">
         <v>0</v>
@@ -33519,7 +33519,7 @@
         <v>0</v>
       </c>
       <c r="M49">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N49">
         <v>0</v>
@@ -33611,7 +33611,7 @@
         <v>0</v>
       </c>
       <c r="M50">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N50">
         <v>0</v>
@@ -33703,7 +33703,7 @@
         <v>0</v>
       </c>
       <c r="M51">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N51">
         <v>0</v>

</xml_diff>